<commit_message>
Fix the cash-basis regime check and label the workbook as a reconciliation
Chow's audit of the workbook found three points, and all three are applied:
- Appraisal!C22 read the confirmed-basis break-even attendance. It now reads the cash-basis value (C21), so the cash regime check tests its own basis. Both checks read OK, and the values are unchanged.
- The sensitivity chart showed only the confirmed basis. It now also shows the cash-cost proxy series.
- The title and a limits note now say the workbook is a legacy-model reconciliation with a cash-cost proxy. It is not a complete Financial Appraisal: cash tax, replacement capex, working capital and the park-only capex and revenue boundary are not modelled, and the depreciation treatment is pending the team's decision.

No input values changed. Recalculated: confirmed NPV -280.94, cash NPV -259.42, all 26 sensitivity cases within 2e-13 of the model.

Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seminar/workbook/Phase1_financial_appraisal.xlsx
+++ b/seminar/workbook/Phase1_financial_appraisal.xlsx
@@ -443,7 +443,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Operator NPV by sensitivity case, confirmed basis, THB bn</a:t>
+              <a:t>Operator NPV by sensitivity case, THB bn (confirmed and cash-cost proxy)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -474,6 +474,30 @@
           <val>
             <numRef>
               <f>'Appraisal'!$G$57:$G$82</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Appraisal'!H56</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Appraisal'!$A$57:$A$82</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Appraisal'!$H$57:$H$82</f>
             </numRef>
           </val>
         </ser>
@@ -5908,7 +5932,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Operator financial appraisal, base case (THB billion unless stated)</t>
+          <t>Operator financial appraisal: legacy-model reconciliation and cash-cost proxy (base case, THB billion unless stated)</t>
         </is>
       </c>
     </row>
@@ -5919,6 +5943,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Limits: not a complete Financial Appraisal. The cash basis is a proxy from Hong Kong Disneyland FY2025 accounts. Not modelled: cash tax, replacement capex, working capital, and the park-only capex and revenue boundary. The depreciation treatment is pending the team decision.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -6153,7 +6184,7 @@
         <v/>
       </c>
       <c r="C22">
-        <f>IF(B21*B11&gt;=B12,"OK","CHECK")</f>
+        <f>IF(C21*B11&gt;=B12,"OK","CHECK")</f>
         <v/>
       </c>
     </row>

</xml_diff>